<commit_message>
Se agrego la columna bodega al excel.
</commit_message>
<xml_diff>
--- a/DiamDev.Give.UI/Content/Formatos/ProductosCargaMasiva.xlsx
+++ b/DiamDev.Give.UI/Content/Formatos/ProductosCargaMasiva.xlsx
@@ -5,17 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Inventory\DiamDev.Give.UI\Content\Formatos\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7530"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4455"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$L$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$M$3</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
   <si>
     <t>ID</t>
   </si>
@@ -78,6 +78,15 @@
   </si>
   <si>
     <t>CHALINA TALLA UNICA</t>
+  </si>
+  <si>
+    <t>BODEGA</t>
+  </si>
+  <si>
+    <t>Z10</t>
+  </si>
+  <si>
+    <t>CAYALA</t>
   </si>
 </sst>
 </file>
@@ -471,24 +480,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.85546875" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.140625" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="9.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="12.85546875" style="3"/>
+    <col min="3" max="3" width="18.85546875" style="3" customWidth="1"/>
+    <col min="4" max="4" width="31" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="9.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="12.85546875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -496,113 +506,122 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="4">
         <v>20170111240</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="9">
+      <c r="F2" s="9">
         <v>1</v>
       </c>
-      <c r="F2" s="5">
+      <c r="G2" s="5">
         <v>92</v>
       </c>
-      <c r="G2" s="5">
+      <c r="H2" s="5">
         <v>130</v>
       </c>
-      <c r="H2" s="4">
+      <c r="I2" s="4">
         <v>2</v>
       </c>
-      <c r="I2" s="4">
+      <c r="J2" s="4">
         <v>3</v>
       </c>
-      <c r="J2" s="7">
-        <f t="shared" ref="J2:J3" si="0">G2-F2</f>
+      <c r="K2" s="7">
+        <f t="shared" ref="K2:K3" si="0">H2-G2</f>
         <v>38</v>
       </c>
-      <c r="K2" s="6">
-        <f t="shared" ref="K2" si="1">J3/G2</f>
+      <c r="L2" s="6">
+        <f t="shared" ref="L2" si="1">K3/H2</f>
         <v>0.61538461538461542</v>
       </c>
-      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="4">
         <v>20170303041</v>
       </c>
       <c r="B3" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="9">
+      <c r="F3" s="9">
         <v>1</v>
       </c>
-      <c r="F3" s="5">
+      <c r="G3" s="5">
         <v>200</v>
       </c>
-      <c r="G3" s="5">
+      <c r="H3" s="5">
         <v>280</v>
       </c>
-      <c r="H3" s="4">
+      <c r="I3" s="4">
         <v>2</v>
       </c>
-      <c r="I3" s="4">
+      <c r="J3" s="4">
         <v>3</v>
       </c>
-      <c r="J3" s="7">
+      <c r="K3" s="7">
         <f t="shared" si="0"/>
         <v>80</v>
       </c>
-      <c r="K3" s="6">
-        <f>J3/G3</f>
+      <c r="L3" s="6">
+        <f>K3/H3</f>
         <v>0.2857142857142857</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="M3" s="4" t="s">
         <v>11</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L3"/>
+  <autoFilter ref="A1:M3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="260" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
se carga el excel como un json
</commit_message>
<xml_diff>
--- a/DiamDev.Give.UI/Content/Formatos/ProductosCargaMasiva.xlsx
+++ b/DiamDev.Give.UI/Content/Formatos/ProductosCargaMasiva.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>ID</t>
   </si>
@@ -87,6 +87,9 @@
   </si>
   <si>
     <t>CAYALA</t>
+  </si>
+  <si>
+    <t>MODIFICACION</t>
   </si>
 </sst>
 </file>
@@ -183,9 +186,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -483,140 +485,143 @@
   <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.85546875" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.85546875" style="3" customWidth="1"/>
-    <col min="4" max="4" width="31" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="9.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="12.85546875" style="3"/>
+    <col min="1" max="1" width="12.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.85546875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="31" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="9.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="12.85546875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="4">
+      <c r="A2" s="3">
         <v>20170111240</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="9">
+      <c r="F2" s="8">
         <v>1</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="4">
         <v>92</v>
       </c>
-      <c r="H2" s="5">
+      <c r="H2" s="4">
         <v>130</v>
       </c>
-      <c r="I2" s="4">
+      <c r="I2" s="3">
         <v>2</v>
       </c>
-      <c r="J2" s="4">
+      <c r="J2" s="3">
         <v>3</v>
       </c>
-      <c r="K2" s="7">
+      <c r="K2" s="6">
         <f t="shared" ref="K2:K3" si="0">H2-G2</f>
         <v>38</v>
       </c>
-      <c r="L2" s="6">
+      <c r="L2" s="5">
         <f t="shared" ref="L2" si="1">K3/H2</f>
         <v>0.61538461538461542</v>
       </c>
-      <c r="M2" s="4"/>
+      <c r="M2" s="3"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" s="4">
+      <c r="A3" s="3">
         <v>20170303041</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="8">
         <v>1</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="4">
         <v>200</v>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="4">
         <v>280</v>
       </c>
-      <c r="I3" s="4">
+      <c r="I3" s="3">
         <v>2</v>
       </c>
-      <c r="J3" s="4">
+      <c r="J3" s="3">
         <v>3</v>
       </c>
-      <c r="K3" s="7">
+      <c r="K3" s="6">
         <f t="shared" si="0"/>
         <v>80</v>
       </c>
-      <c r="L3" s="6">
+      <c r="L3" s="5">
         <f>K3/H3</f>
         <v>0.2857142857142857</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="M3" s="3" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>